<commit_message>
Update tripling diagnostics and risk model
</commit_message>
<xml_diff>
--- a/tripling_beta/tripling.xlsx
+++ b/tripling_beta/tripling.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Documents\GitHub\tripling_beta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Documents\GitHub\GIPT\tripling_beta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EEE3D90-E130-4C21-BDD3-EC033DF9F5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD457CC-2C93-4D4E-B43E-71A6A41D2259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{64387DDE-4ECD-4D35-9D9B-650204D19CA6}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="30">
   <si>
     <t>Historical annual capacity additions</t>
   </si>
@@ -82,6 +82,54 @@
   </si>
   <si>
     <t>Cumulative</t>
+  </si>
+  <si>
+    <t>Total RE</t>
+  </si>
+  <si>
+    <t>Total RE additions</t>
+  </si>
+  <si>
+    <t>Total solar PV</t>
+  </si>
+  <si>
+    <t>Total wind</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Total capacity</t>
+  </si>
+  <si>
+    <t>Renewables</t>
+  </si>
+  <si>
+    <t>Solar PV</t>
+  </si>
+  <si>
+    <t>Bioenergy</t>
+  </si>
+  <si>
+    <t>of which BECCS</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>CSP</t>
+  </si>
+  <si>
+    <t>Geothermal</t>
+  </si>
+  <si>
+    <t>Marine</t>
+  </si>
+  <si>
+    <t>Total hydro</t>
+  </si>
+  <si>
+    <t>Total Other</t>
   </si>
 </sst>
 </file>
@@ -163,7 +211,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -172,10 +220,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -183,6 +231,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1123,72 +1177,72 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>additions!$C$32:$C$52</c:f>
+              <c:f>additions!$K$32:$K$52</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>3.8759999999999999</c:v>
+                  <c:v>33.489999999999903</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.2735000000000003</c:v>
+                  <c:v>60.1799999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.2650000000000006</c:v>
+                  <c:v>85.739500000000007</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>19.702999999999999</c:v>
+                  <c:v>118.506999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22.9755</c:v>
+                  <c:v>155.91550000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>31.263000000000002</c:v>
+                  <c:v>203.26899999999901</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>52.6829999999999</c:v>
+                  <c:v>273.69150000000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>59.219499999999996</c:v>
+                  <c:v>365.8655</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>54.340499999999999</c:v>
+                  <c:v>457.945999999999</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>64.6935</c:v>
+                  <c:v>562.27499999999998</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>71.468000000000004</c:v>
+                  <c:v>689.63049999999998</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>75.471500000000006</c:v>
+                  <c:v>830.43299999999999</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>92.054999999999893</c:v>
+                  <c:v>1019.44749999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>200.4385</c:v>
+                  <c:v>1379.4480000000001</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>275.671999999999</c:v>
+                  <c:v>1836.4675</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>305.71949999999998</c:v>
+                  <c:v>2745</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>359.04799121639996</c:v>
+                  <c:v>3362.6250000000005</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>399.65835743279996</c:v>
+                  <c:v>4085.5893750000009</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>440.26872364919996</c:v>
+                  <c:v>4841.423409375001</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>480.87908986559989</c:v>
+                  <c:v>5688.6725060156268</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>521.48945608200029</c:v>
+                  <c:v>6699</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4500,10 +4554,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{618F5C34-951E-4D38-B3E7-3ECB10372AC8}">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="15" width="7.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -4511,8 +4568,26 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>2015</v>
       </c>
@@ -4527,8 +4602,11 @@
       <c r="E2">
         <v>1867</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I2" s="1">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2016</v>
       </c>
@@ -4544,8 +4622,11 @@
         <f>E2+D3</f>
         <v>2032.24</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I3" s="1">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2017</v>
       </c>
@@ -4561,8 +4642,11 @@
         <f t="shared" ref="E4:E16" si="1">E3+D4</f>
         <v>2196.9899999999998</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I4" s="1">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2018</v>
       </c>
@@ -4578,8 +4662,11 @@
         <f t="shared" si="1"/>
         <v>2361.2599999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I5" s="1">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>2019</v>
       </c>
@@ -4595,8 +4682,11 @@
         <f t="shared" si="1"/>
         <v>2540.12</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6" s="1">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>2020</v>
       </c>
@@ -4612,8 +4702,11 @@
         <f t="shared" si="1"/>
         <v>2804.0499999999997</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I7" s="1">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>2021</v>
       </c>
@@ -4629,8 +4722,11 @@
         <f t="shared" si="1"/>
         <v>3065.29</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I8" s="1">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>2022</v>
       </c>
@@ -4646,8 +4742,26 @@
         <f t="shared" si="1"/>
         <v>3371.76</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9" s="1">
+        <v>2022</v>
+      </c>
+      <c r="K9">
+        <v>3684</v>
+      </c>
+      <c r="L9">
+        <v>1185</v>
+      </c>
+      <c r="M9">
+        <v>899</v>
+      </c>
+      <c r="N9">
+        <v>1398</v>
+      </c>
+      <c r="O9">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>2023</v>
       </c>
@@ -4663,8 +4777,30 @@
         <f t="shared" si="1"/>
         <v>3858.1600000000003</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I10" s="1">
+        <v>2023</v>
+      </c>
+      <c r="J10">
+        <f>K10-K9</f>
+        <v>562</v>
+      </c>
+      <c r="K10">
+        <v>4246</v>
+      </c>
+      <c r="L10">
+        <v>1610</v>
+      </c>
+      <c r="M10">
+        <v>1016</v>
+      </c>
+      <c r="N10">
+        <v>1410</v>
+      </c>
+      <c r="O10">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>2024</v>
       </c>
@@ -4680,8 +4816,34 @@
         <f t="shared" si="1"/>
         <v>4440.16</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I11" s="1">
+        <v>2024</v>
+      </c>
+      <c r="J11">
+        <f>K11-K10</f>
+        <v>689</v>
+      </c>
+      <c r="K11">
+        <v>4935</v>
+      </c>
+      <c r="L11">
+        <v>2164</v>
+      </c>
+      <c r="M11">
+        <v>1131</v>
+      </c>
+      <c r="N11">
+        <v>1437</v>
+      </c>
+      <c r="O11">
+        <v>205</v>
+      </c>
+      <c r="P11">
+        <f>SUM(N11:O11)</f>
+        <v>1642</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>2025</v>
       </c>
@@ -4696,11 +4858,47 @@
         <f t="shared" si="1"/>
         <v>5132.16</v>
       </c>
-      <c r="I12">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I12" s="1">
+        <v>2025</v>
+      </c>
+      <c r="J12">
+        <f>K12-K11</f>
+        <v>799.00000000000091</v>
+      </c>
+      <c r="K12">
+        <f>SUM(L12:O12)</f>
+        <v>5734.0000000000009</v>
+      </c>
+      <c r="L12">
+        <f>L11+605</f>
+        <v>2769</v>
+      </c>
+      <c r="M12">
+        <f>M11+159</f>
+        <v>1290</v>
+      </c>
+      <c r="N12" s="2">
+        <f>(N11/SUM(N11:O11))*(P12-P11)+N11</f>
+        <v>1465.880024360536</v>
+      </c>
+      <c r="O12" s="2">
+        <f>(O11/SUM(N11:O11))*(P12-P11)+O11</f>
+        <v>209.11997563946406</v>
+      </c>
+      <c r="P12">
+        <f>SUM(N11:O11)+33</f>
+        <v>1675</v>
+      </c>
+      <c r="R12">
+        <f>L12*0.85</f>
+        <v>2353.65</v>
+      </c>
+      <c r="S12">
+        <f>L12-R12</f>
+        <v>415.34999999999991</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>2026</v>
       </c>
@@ -4716,8 +4914,11 @@
         <f>E12+D13</f>
         <v>5982.16</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I13" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>2027</v>
       </c>
@@ -4733,8 +4934,11 @@
         <f t="shared" si="1"/>
         <v>6967.16</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I14" s="1">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>2028</v>
       </c>
@@ -4750,8 +4954,11 @@
         <f t="shared" si="1"/>
         <v>8117.16</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I15" s="1">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>2029</v>
       </c>
@@ -4767,8 +4974,11 @@
         <f t="shared" si="1"/>
         <v>9452.16</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I16" s="1">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>2030</v>
       </c>
@@ -4784,53 +4994,465 @@
         <f>E16+D17</f>
         <v>11007.16</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17" s="1">
+        <v>2030</v>
+      </c>
+      <c r="K17">
+        <v>11495</v>
+      </c>
+      <c r="L17">
+        <v>6699</v>
+      </c>
+      <c r="M17">
+        <v>2731</v>
+      </c>
+      <c r="N17">
+        <v>1697</v>
+      </c>
+      <c r="O17">
+        <v>383</v>
+      </c>
+      <c r="R17">
+        <f>L17*0.85</f>
+        <v>5694.15</v>
+      </c>
+      <c r="S17">
+        <f>L17-R17</f>
+        <v>1004.8500000000004</v>
+      </c>
+      <c r="T17">
+        <f>K17-S17</f>
+        <v>10490.15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C19">
         <f>SUM(C13:C17)</f>
         <v>5875</v>
       </c>
-      <c r="G19">
-        <f>E17-E12</f>
-        <v>5875</v>
-      </c>
-      <c r="H19">
-        <f>G19/5</f>
-        <v>1175</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C20">
-        <f>C19-4745</f>
-        <v>1130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K19">
+        <f>K17-K12</f>
+        <v>5760.9999999999991</v>
+      </c>
+      <c r="M19">
+        <f>SUM(L17:N17)</f>
+        <v>11127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K20">
+        <f>K19-5093</f>
+        <v>667.99999999999909</v>
+      </c>
+      <c r="M20" s="2">
+        <f>M19-SUM(L12:N12)</f>
+        <v>5602.1199756394635</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="M21" s="2">
+        <f>M20-5093</f>
+        <v>509.11997563946352</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C22">
         <v>5093.5</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C23">
         <f>C19-C22</f>
         <v>781.5</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I23" t="s">
+        <v>18</v>
+      </c>
+      <c r="J23">
+        <v>2010</v>
+      </c>
+      <c r="K23">
+        <v>2023</v>
+      </c>
+      <c r="L23">
+        <v>2024</v>
+      </c>
+      <c r="M23">
+        <v>2035</v>
+      </c>
+      <c r="O23" t="s">
+        <v>18</v>
+      </c>
+      <c r="P23">
+        <v>2010</v>
+      </c>
+      <c r="Q23">
+        <v>2022</v>
+      </c>
+      <c r="R23">
+        <v>2023</v>
+      </c>
+      <c r="S23">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I24" t="s">
+        <v>19</v>
+      </c>
+      <c r="J24">
+        <v>5254</v>
+      </c>
+      <c r="K24">
+        <v>9441</v>
+      </c>
+      <c r="L24">
+        <v>10249</v>
+      </c>
+      <c r="M24">
+        <v>26552</v>
+      </c>
+      <c r="O24" t="s">
+        <v>19</v>
+      </c>
+      <c r="P24">
+        <v>5259</v>
+      </c>
+      <c r="Q24">
+        <v>8768</v>
+      </c>
+      <c r="R24">
+        <v>9436</v>
+      </c>
+      <c r="S24">
+        <v>17093</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I25" t="s">
+        <v>20</v>
+      </c>
+      <c r="J25">
+        <v>1332</v>
+      </c>
+      <c r="K25">
+        <v>4249</v>
+      </c>
+      <c r="L25">
+        <v>4935</v>
+      </c>
+      <c r="M25">
+        <v>19601</v>
+      </c>
+      <c r="O25" t="s">
+        <v>20</v>
+      </c>
+      <c r="P25">
+        <v>1334</v>
+      </c>
+      <c r="Q25">
+        <v>3684</v>
+      </c>
+      <c r="R25">
+        <v>4246</v>
+      </c>
+      <c r="S25">
+        <v>11495</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
+      <c r="I26" t="s">
+        <v>21</v>
+      </c>
+      <c r="J26">
+        <v>40</v>
+      </c>
+      <c r="K26">
+        <v>1625</v>
+      </c>
+      <c r="L26">
+        <v>2164</v>
+      </c>
+      <c r="M26">
+        <v>12499</v>
+      </c>
+      <c r="O26" t="s">
+        <v>21</v>
+      </c>
+      <c r="P26">
+        <v>40</v>
+      </c>
+      <c r="Q26">
+        <v>1185</v>
+      </c>
+      <c r="R26">
+        <v>1610</v>
+      </c>
+      <c r="S26">
+        <v>6699</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="I27" t="s">
+        <v>7</v>
+      </c>
+      <c r="J27">
+        <v>181</v>
+      </c>
+      <c r="K27">
+        <v>1016</v>
+      </c>
+      <c r="L27">
+        <v>1131</v>
+      </c>
+      <c r="M27">
+        <v>4494</v>
+      </c>
+      <c r="O27" t="s">
+        <v>7</v>
+      </c>
+      <c r="P27">
+        <v>181</v>
+      </c>
+      <c r="Q27">
+        <v>899</v>
+      </c>
+      <c r="R27">
+        <v>1015</v>
+      </c>
+      <c r="S27">
+        <v>2731</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="I28" t="s">
+        <v>11</v>
+      </c>
+      <c r="J28">
+        <v>1026</v>
+      </c>
+      <c r="K28">
+        <v>1410</v>
+      </c>
+      <c r="L28">
+        <v>1437</v>
+      </c>
+      <c r="M28">
+        <v>2037</v>
+      </c>
+      <c r="O28" t="s">
+        <v>11</v>
+      </c>
+      <c r="P28">
+        <v>1028</v>
+      </c>
+      <c r="Q28">
+        <v>1398</v>
+      </c>
+      <c r="R28">
+        <v>1411</v>
+      </c>
+      <c r="S28">
+        <v>1697</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="I29" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29">
+        <v>73</v>
+      </c>
+      <c r="K29">
+        <v>175</v>
+      </c>
+      <c r="L29">
+        <v>181</v>
+      </c>
+      <c r="M29">
+        <v>413</v>
+      </c>
+      <c r="O29" t="s">
+        <v>22</v>
+      </c>
+      <c r="P29">
+        <v>74</v>
+      </c>
+      <c r="Q29">
+        <v>180</v>
+      </c>
+      <c r="R29">
+        <v>188</v>
+      </c>
+      <c r="S29">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="I30" t="s">
+        <v>23</v>
+      </c>
+      <c r="J30" t="s">
+        <v>24</v>
+      </c>
+      <c r="K30" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" t="s">
+        <v>24</v>
+      </c>
+      <c r="M30">
+        <v>63</v>
+      </c>
+      <c r="O30" t="s">
+        <v>23</v>
+      </c>
+      <c r="P30" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>24</v>
+      </c>
+      <c r="R30" t="s">
+        <v>24</v>
+      </c>
+      <c r="S30">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="I31" t="s">
+        <v>25</v>
+      </c>
+      <c r="J31">
+        <v>1</v>
+      </c>
+      <c r="K31">
+        <v>7</v>
+      </c>
+      <c r="L31">
+        <v>8</v>
+      </c>
+      <c r="M31">
+        <v>91</v>
+      </c>
+      <c r="O31" t="s">
+        <v>25</v>
+      </c>
+      <c r="P31">
+        <v>1</v>
+      </c>
+      <c r="Q31">
+        <v>6</v>
+      </c>
+      <c r="R31">
+        <v>7</v>
+      </c>
+      <c r="S31">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="I32" t="s">
+        <v>26</v>
+      </c>
+      <c r="J32">
+        <v>10</v>
+      </c>
+      <c r="K32">
+        <v>15</v>
+      </c>
+      <c r="L32">
+        <v>15</v>
+      </c>
+      <c r="M32">
+        <v>57</v>
+      </c>
+      <c r="O32" t="s">
+        <v>26</v>
+      </c>
+      <c r="P32">
+        <v>10</v>
+      </c>
+      <c r="Q32">
+        <v>15</v>
+      </c>
+      <c r="R32">
+        <v>15</v>
+      </c>
+      <c r="S32">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I33" t="s">
+        <v>27</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>1</v>
+      </c>
+      <c r="L33">
+        <v>1</v>
+      </c>
+      <c r="M33">
+        <v>11</v>
+      </c>
+      <c r="O33" t="s">
+        <v>27</v>
+      </c>
+      <c r="P33">
+        <v>0</v>
+      </c>
+      <c r="Q33">
+        <v>1</v>
+      </c>
+      <c r="R33">
+        <v>1</v>
+      </c>
+      <c r="S33">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I42" s="11"/>
+      <c r="J42" s="11"/>
+    </row>
+    <row r="43" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I43" s="11"/>
+      <c r="J43" s="11"/>
+    </row>
+    <row r="44" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I44" s="11"/>
+      <c r="J44" s="11"/>
+    </row>
+    <row r="45" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I45" s="11"/>
+      <c r="J45" s="11"/>
+    </row>
+    <row r="46" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I46" s="11"/>
+      <c r="J46" s="11"/>
+    </row>
+    <row r="47" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I47" s="11"/>
+      <c r="J47" s="11"/>
+    </row>
+    <row r="48" spans="9:19" x14ac:dyDescent="0.25">
+      <c r="I48" s="11"/>
+      <c r="J48" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4839,33 +5461,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956A7829-92DD-491D-9D03-157647D17055}">
-  <dimension ref="A4:S84"/>
+  <dimension ref="A4:U84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="K4" s="6" t="s">
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="K4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
@@ -5437,7 +6059,7 @@
         <v>1186.125</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2020</v>
       </c>
@@ -5489,7 +6111,7 @@
         <v>1421.6704999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2021</v>
       </c>
@@ -5541,7 +6163,7 @@
         <v>1655.2930000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2022</v>
       </c>
@@ -5592,8 +6214,9 @@
         <f t="shared" si="2"/>
         <v>1920.43749999999</v>
       </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T19" s="2"/>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2023</v>
       </c>
@@ -5644,8 +6267,9 @@
         <f t="shared" si="2"/>
         <v>2395.018</v>
       </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T20" s="2"/>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2024</v>
       </c>
@@ -5703,8 +6327,9 @@
         <f>R21+K21+N21</f>
         <v>4609.1374999999998</v>
       </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T21" s="2"/>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2025</v>
       </c>
@@ -5760,11 +6385,12 @@
         <v>1712.8333333333333</v>
       </c>
       <c r="S22" s="2">
-        <f t="shared" ref="S22:S27" si="3">R22+K22+N22</f>
+        <f>R22+K22+N22</f>
         <v>5393.3033333333333</v>
       </c>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T22" s="2"/>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2026</v>
       </c>
@@ -5773,27 +6399,27 @@
         <v>860.77399999999989</v>
       </c>
       <c r="C23" s="2">
-        <f t="shared" ref="C23:G27" si="4">L23-L22</f>
+        <f t="shared" ref="C23:G27" si="3">L23-L22</f>
         <v>537.42581999999993</v>
       </c>
       <c r="D23" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>323.33968000000004</v>
       </c>
       <c r="E23" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>289.13200000000006</v>
       </c>
       <c r="F23" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>262.25423999999998</v>
       </c>
       <c r="G23" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>26.877760000000009</v>
       </c>
       <c r="H23" s="2">
-        <f t="shared" ref="H23:H27" si="5">R23-R22</f>
+        <f t="shared" ref="H23:H27" si="4">R23-R22</f>
         <v>70.833333333333258</v>
       </c>
       <c r="I23" s="2"/>
@@ -5829,15 +6455,23 @@
         <v>4830.3760000000002</v>
       </c>
       <c r="R23" s="2">
-        <f t="shared" ref="R23:R26" si="6">($R$27-$R$21)/6+R22</f>
+        <f t="shared" ref="R23:R26" si="5">($R$27-$R$21)/6+R22</f>
         <v>1783.6666666666665</v>
       </c>
       <c r="S23" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="S23:S27" si="6">R23+K23+N23</f>
         <v>6614.0426666666663</v>
       </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T23" s="2">
+        <f>S23-S22</f>
+        <v>1220.739333333333</v>
+      </c>
+      <c r="U23" s="2">
+        <f>B48+E48+H23</f>
+        <v>928.29900423911636</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2027</v>
       </c>
@@ -5846,19 +6480,19 @@
         <v>860.77399999999989</v>
       </c>
       <c r="C24" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>499.24891999999977</v>
       </c>
       <c r="D24" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>361.52508000000012</v>
       </c>
       <c r="E24" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>289.13200000000006</v>
       </c>
       <c r="F24" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>266.00144000000023</v>
       </c>
       <c r="G24" s="2">
@@ -5866,7 +6500,7 @@
         <v>23.130559999999832</v>
       </c>
       <c r="H24" s="2">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>70.833333333333258</v>
       </c>
       <c r="I24" s="2"/>
@@ -5902,15 +6536,23 @@
         <v>5980.2820000000002</v>
       </c>
       <c r="R24" s="2">
+        <f t="shared" si="5"/>
+        <v>1854.4999999999998</v>
+      </c>
+      <c r="S24" s="2">
         <f t="shared" si="6"/>
-        <v>1854.4999999999998</v>
-      </c>
-      <c r="S24" s="2">
-        <f t="shared" si="3"/>
         <v>7834.7820000000002</v>
       </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T24" s="2">
+        <f t="shared" ref="T23:T26" si="14">S24-S23</f>
+        <v>1220.7393333333339</v>
+      </c>
+      <c r="U24" s="2">
+        <f t="shared" ref="U24:U27" si="15">B49+E49+H24</f>
+        <v>1072.4421751448995</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2028</v>
       </c>
@@ -5919,27 +6561,27 @@
         <v>860.77400000000034</v>
       </c>
       <c r="C25" s="2">
+        <f t="shared" si="3"/>
+        <v>499.24892000000045</v>
+      </c>
+      <c r="D25" s="2">
+        <f t="shared" si="3"/>
+        <v>361.52507999999989</v>
+      </c>
+      <c r="E25" s="2">
+        <f t="shared" si="3"/>
+        <v>289.13199999999983</v>
+      </c>
+      <c r="F25" s="2">
+        <f t="shared" si="3"/>
+        <v>266.00143999999977</v>
+      </c>
+      <c r="G25" s="2">
+        <f t="shared" si="3"/>
+        <v>23.13056000000006</v>
+      </c>
+      <c r="H25" s="2">
         <f t="shared" si="4"/>
-        <v>499.24892000000045</v>
-      </c>
-      <c r="D25" s="2">
-        <f t="shared" si="4"/>
-        <v>361.52507999999989</v>
-      </c>
-      <c r="E25" s="2">
-        <f t="shared" si="4"/>
-        <v>289.13199999999983</v>
-      </c>
-      <c r="F25" s="2">
-        <f t="shared" si="4"/>
-        <v>266.00143999999977</v>
-      </c>
-      <c r="G25" s="2">
-        <f t="shared" si="4"/>
-        <v>23.13056000000006</v>
-      </c>
-      <c r="H25" s="2">
-        <f t="shared" si="5"/>
         <v>70.833333333333258</v>
       </c>
       <c r="I25" s="2"/>
@@ -5975,15 +6617,23 @@
         <v>7130.1880000000001</v>
       </c>
       <c r="R25" s="2">
+        <f t="shared" si="5"/>
+        <v>1925.333333333333</v>
+      </c>
+      <c r="S25" s="2">
         <f t="shared" si="6"/>
-        <v>1925.333333333333</v>
-      </c>
-      <c r="S25" s="2">
-        <f t="shared" si="3"/>
         <v>9055.521333333334</v>
       </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T25" s="2">
+        <f t="shared" si="14"/>
+        <v>1220.7393333333339</v>
+      </c>
+      <c r="U25" s="2">
+        <f t="shared" si="15"/>
+        <v>1216.5853460506826</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2029</v>
       </c>
@@ -5992,27 +6642,27 @@
         <v>860.77400000000034</v>
       </c>
       <c r="C26" s="2">
+        <f t="shared" si="3"/>
+        <v>499.24892</v>
+      </c>
+      <c r="D26" s="2">
+        <f t="shared" si="3"/>
+        <v>361.52508000000034</v>
+      </c>
+      <c r="E26" s="2">
+        <f t="shared" si="3"/>
+        <v>289.13200000000006</v>
+      </c>
+      <c r="F26" s="2">
+        <f t="shared" si="3"/>
+        <v>266.00144</v>
+      </c>
+      <c r="G26" s="2">
+        <f t="shared" si="3"/>
+        <v>23.13056000000006</v>
+      </c>
+      <c r="H26" s="2">
         <f t="shared" si="4"/>
-        <v>499.24892</v>
-      </c>
-      <c r="D26" s="2">
-        <f t="shared" si="4"/>
-        <v>361.52508000000034</v>
-      </c>
-      <c r="E26" s="2">
-        <f t="shared" si="4"/>
-        <v>289.13200000000006</v>
-      </c>
-      <c r="F26" s="2">
-        <f t="shared" si="4"/>
-        <v>266.00144</v>
-      </c>
-      <c r="G26" s="2">
-        <f t="shared" si="4"/>
-        <v>23.13056000000006</v>
-      </c>
-      <c r="H26" s="2">
-        <f t="shared" si="5"/>
         <v>70.833333333333258</v>
       </c>
       <c r="I26" s="2"/>
@@ -6048,15 +6698,23 @@
         <v>8280.094000000001</v>
       </c>
       <c r="R26" s="2">
+        <f t="shared" si="5"/>
+        <v>1996.1666666666663</v>
+      </c>
+      <c r="S26" s="2">
         <f t="shared" si="6"/>
-        <v>1996.1666666666663</v>
-      </c>
-      <c r="S26" s="2">
-        <f t="shared" si="3"/>
         <v>10276.260666666667</v>
       </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T26" s="2">
+        <f t="shared" si="14"/>
+        <v>1220.739333333333</v>
+      </c>
+      <c r="U26" s="2">
+        <f t="shared" si="15"/>
+        <v>1360.7285169564655</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2030</v>
       </c>
@@ -6065,27 +6723,27 @@
         <v>860.77399999999943</v>
       </c>
       <c r="C27" s="2">
+        <f t="shared" si="3"/>
+        <v>499.24891999999954</v>
+      </c>
+      <c r="D27" s="2">
+        <f t="shared" si="3"/>
+        <v>361.52507999999989</v>
+      </c>
+      <c r="E27" s="2">
+        <f t="shared" si="3"/>
+        <v>289.13200000000006</v>
+      </c>
+      <c r="F27" s="2">
+        <f t="shared" si="3"/>
+        <v>266.00144</v>
+      </c>
+      <c r="G27" s="2">
+        <f t="shared" si="3"/>
+        <v>23.13056000000006</v>
+      </c>
+      <c r="H27" s="2">
         <f t="shared" si="4"/>
-        <v>499.24891999999954</v>
-      </c>
-      <c r="D27" s="2">
-        <f t="shared" si="4"/>
-        <v>361.52507999999989</v>
-      </c>
-      <c r="E27" s="2">
-        <f t="shared" si="4"/>
-        <v>289.13200000000006</v>
-      </c>
-      <c r="F27" s="2">
-        <f t="shared" si="4"/>
-        <v>266.00144</v>
-      </c>
-      <c r="G27" s="2">
-        <f t="shared" si="4"/>
-        <v>23.13056000000006</v>
-      </c>
-      <c r="H27" s="2">
-        <f t="shared" si="5"/>
         <v>70.833333333333712</v>
       </c>
       <c r="I27" s="2"/>
@@ -6123,11 +6781,25 @@
         <v>2067</v>
       </c>
       <c r="S27" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>11497</v>
       </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T27" s="2">
+        <f>S27-S26</f>
+        <v>1220.739333333333</v>
+      </c>
+      <c r="U27" s="2">
+        <f t="shared" si="15"/>
+        <v>1504.8716878622488</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="R29" s="2">
+        <f>R27-R22</f>
+        <v>354.16666666666674</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B30" s="8" t="s">
         <v>9</v>
       </c>
@@ -6145,7 +6817,7 @@
       <c r="O30" s="9"/>
       <c r="P30" s="9"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>2</v>
       </c>
@@ -6183,7 +6855,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2010</v>
       </c>
@@ -6245,7 +6917,7 @@
         <v>17.416499999999999</v>
       </c>
       <c r="E33" s="2">
-        <f t="shared" ref="E33:E47" si="14">SUM(F33:G33)</f>
+        <f t="shared" ref="E33:E47" si="16">SUM(F33:G33)</f>
         <v>39.11</v>
       </c>
       <c r="F33" s="2">
@@ -6269,7 +6941,7 @@
         <v>44.157499999999999</v>
       </c>
       <c r="N33" s="2">
-        <f t="shared" ref="N33:N47" si="15">SUM(O33:P33)</f>
+        <f t="shared" ref="N33:N47" si="17">SUM(O33:P33)</f>
         <v>220.36</v>
       </c>
       <c r="O33" s="2">
@@ -6293,7 +6965,7 @@
         <v>16.286000000000001</v>
       </c>
       <c r="E34" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>46.919999999999995</v>
       </c>
       <c r="F34" s="2">
@@ -6317,7 +6989,7 @@
         <v>60.4435</v>
       </c>
       <c r="N34" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>267.28000000000003</v>
       </c>
       <c r="O34" s="2">
@@ -6341,7 +7013,7 @@
         <v>13.064499999999899</v>
       </c>
       <c r="E35" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>32.92</v>
       </c>
       <c r="F35" s="2">
@@ -6365,7 +7037,7 @@
         <v>73.507999999999996</v>
       </c>
       <c r="N35" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>300.19</v>
       </c>
       <c r="O35" s="2">
@@ -6389,7 +7061,7 @@
         <v>14.433</v>
       </c>
       <c r="E36" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>49.6</v>
       </c>
       <c r="F36" s="2">
@@ -6413,7 +7085,7 @@
         <v>87.940999999999903</v>
       </c>
       <c r="N36" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>349.8</v>
       </c>
       <c r="O36" s="2">
@@ -6437,7 +7109,7 @@
         <v>16.090499999999999</v>
       </c>
       <c r="E37" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>65.59</v>
       </c>
       <c r="F37" s="2">
@@ -6461,7 +7133,7 @@
         <v>104.03149999999999</v>
       </c>
       <c r="N37" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>415.39</v>
       </c>
       <c r="O37" s="2">
@@ -6485,7 +7157,7 @@
         <v>17.7395</v>
       </c>
       <c r="E38" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>52.14</v>
       </c>
       <c r="F38" s="2">
@@ -6509,7 +7181,7 @@
         <v>121.77099999999901</v>
       </c>
       <c r="N38" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>467.53</v>
       </c>
       <c r="O38" s="2">
@@ -6533,7 +7205,7 @@
         <v>32.954500000000003</v>
       </c>
       <c r="E39" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>47.63</v>
       </c>
       <c r="F39" s="2">
@@ -6557,7 +7229,7 @@
         <v>154.73399999999901</v>
       </c>
       <c r="N39" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>515.16</v>
       </c>
       <c r="O39" s="2">
@@ -6581,7 +7253,7 @@
         <v>37.7484999999999</v>
       </c>
       <c r="E40" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>49.66</v>
       </c>
       <c r="F40" s="2">
@@ -6605,7 +7277,7 @@
         <v>192.47399999999999</v>
       </c>
       <c r="N40" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>564.82000000000005</v>
       </c>
       <c r="O40" s="2">
@@ -6629,7 +7301,7 @@
         <v>39.626999999999903</v>
       </c>
       <c r="E41" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>59.03</v>
       </c>
       <c r="F41" s="2">
@@ -6653,7 +7325,7 @@
         <v>232.101</v>
       </c>
       <c r="N41" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>623.85</v>
       </c>
       <c r="O41" s="2">
@@ -6677,7 +7349,7 @@
         <v>55.887499999999903</v>
       </c>
       <c r="E42" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>108.19</v>
       </c>
       <c r="F42" s="2">
@@ -6701,7 +7373,7 @@
         <v>287.99700000000001</v>
       </c>
       <c r="N42" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>732.04</v>
       </c>
       <c r="O42" s="2">
@@ -6725,7 +7397,7 @@
         <v>65.331000000000003</v>
       </c>
       <c r="E43" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>92.81</v>
       </c>
       <c r="F43" s="2">
@@ -6749,7 +7421,7 @@
         <v>353.32799999999997</v>
       </c>
       <c r="N43" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>824.86</v>
       </c>
       <c r="O43" s="2">
@@ -6773,7 +7445,7 @@
         <v>96.959499999999906</v>
       </c>
       <c r="E44" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>76.14</v>
       </c>
       <c r="F44" s="2">
@@ -6797,7 +7469,7 @@
         <v>450.287499999999</v>
       </c>
       <c r="N44" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>900.99</v>
       </c>
       <c r="O44" s="2">
@@ -6821,7 +7493,7 @@
         <v>159.56199999999899</v>
       </c>
       <c r="E45" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>114.57</v>
       </c>
       <c r="F45" s="2">
@@ -6845,7 +7517,7 @@
         <v>609.84100000000001</v>
       </c>
       <c r="N45" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1015.5699999999999</v>
       </c>
       <c r="O45" s="2">
@@ -6869,7 +7541,7 @@
         <v>181.3475</v>
       </c>
       <c r="E46" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>115.1</v>
       </c>
       <c r="F46" s="2">
@@ -6893,7 +7565,7 @@
         <v>791.18849999999998</v>
       </c>
       <c r="N46" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1130.67</v>
       </c>
       <c r="O46" s="2">
@@ -6917,7 +7589,7 @@
         <v>252.94299999999899</v>
       </c>
       <c r="E47" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>154.66</v>
       </c>
       <c r="F47" s="2">
@@ -6941,7 +7613,7 @@
         <v>1044.1400000000001</v>
       </c>
       <c r="N47" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1285.3399999999999</v>
       </c>
       <c r="O47" s="2">
@@ -6957,56 +7629,59 @@
       </c>
       <c r="B48" s="2">
         <f>($B$52-$B$47)/5+B47</f>
-        <v>629.90875652</v>
+        <v>648.9954987968747</v>
       </c>
       <c r="C48" s="2">
         <f>B48*0.57</f>
-        <v>359.04799121639996</v>
+        <v>369.92743431421854</v>
       </c>
       <c r="D48" s="2">
         <f>B48-C48</f>
-        <v>270.86076530360003</v>
+        <v>279.06806448265615</v>
       </c>
       <c r="E48" s="2">
         <f>($E$52-$E$47)/5+E47</f>
-        <v>204.47056100352012</v>
+        <v>208.4701721089084</v>
       </c>
       <c r="F48" s="2">
-        <f t="shared" ref="F48:F52" si="16">O48-O47</f>
-        <v>185.45484799999986</v>
+        <f t="shared" ref="F48:F52" si="18">O48-O47</f>
+        <v>182.49856599999998</v>
       </c>
       <c r="G48" s="2">
-        <f t="shared" ref="G48:G52" si="17">P48-P47</f>
-        <v>20.199551999999969</v>
-      </c>
-      <c r="H48" s="2"/>
+        <f t="shared" ref="G48:G52" si="19">P48-P47</f>
+        <v>19.942483999999851</v>
+      </c>
+      <c r="H48" s="2">
+        <f t="shared" ref="H48:H51" si="20">R23-R22</f>
+        <v>70.833333333333258</v>
+      </c>
       <c r="I48" s="4"/>
       <c r="J48">
         <v>2026</v>
       </c>
       <c r="K48" s="2">
         <f>K47*K54</f>
-        <v>3376.35</v>
+        <v>3362.6250000000005</v>
       </c>
       <c r="L48" s="2">
         <f>K48*0.57</f>
-        <v>1924.5194999999999</v>
+        <v>1916.6962500000002</v>
       </c>
       <c r="M48" s="2">
         <f>K48-L48</f>
-        <v>1451.8305</v>
+        <v>1445.9287500000003</v>
       </c>
       <c r="N48" s="2">
         <f>N47*$N$54</f>
-        <v>1490.9943999999998</v>
+        <v>1487.7810499999998</v>
       </c>
       <c r="O48" s="2">
         <f>N48*0.92</f>
-        <v>1371.7148479999998</v>
+        <v>1368.758566</v>
       </c>
       <c r="P48" s="2">
         <f>N48-O48</f>
-        <v>119.27955199999997</v>
+        <v>119.02248399999985</v>
       </c>
       <c r="R48" s="5"/>
     </row>
@@ -7015,57 +7690,60 @@
         <v>2027</v>
       </c>
       <c r="B49" s="2">
-        <f t="shared" ref="B49:B51" si="18">($B$52-$B$47)/5+B48</f>
-        <v>701.15501303999997</v>
+        <f t="shared" ref="B49:B50" si="21">($B$52-$B$47)/5+B48</f>
+        <v>739.32849759374938</v>
       </c>
       <c r="C49" s="2">
         <f>B49*0.57</f>
-        <v>399.65835743279996</v>
+        <v>421.41724362843712</v>
       </c>
       <c r="D49" s="2">
-        <f t="shared" ref="D49:D51" si="19">B49-C49</f>
-        <v>301.49665560720001</v>
+        <f t="shared" ref="D49:D51" si="22">B49-C49</f>
+        <v>317.91125396531226</v>
       </c>
       <c r="E49" s="2">
-        <f t="shared" ref="E49:E51" si="20">($E$52-$E$47)/5+E48</f>
-        <v>254.28112200704027</v>
+        <f t="shared" ref="E49:E51" si="23">($E$52-$E$47)/5+E48</f>
+        <v>262.28034421781678</v>
       </c>
       <c r="F49" s="2">
-        <f t="shared" si="16"/>
-        <v>219.47437568000009</v>
+        <f t="shared" si="18"/>
+        <v>215.57947414499995</v>
       </c>
       <c r="G49" s="2">
-        <f t="shared" si="17"/>
-        <v>19.08472831999984</v>
-      </c>
-      <c r="H49" s="2"/>
+        <f t="shared" si="19"/>
+        <v>18.746041229999946</v>
+      </c>
+      <c r="H49" s="2">
+        <f t="shared" si="20"/>
+        <v>70.833333333333258</v>
+      </c>
       <c r="I49" s="4"/>
       <c r="J49">
         <v>2027</v>
       </c>
       <c r="K49" s="2">
-        <f t="shared" ref="K49:K51" si="21">K48*K55</f>
-        <v>4119.1469999999999</v>
+        <f t="shared" ref="K49:K50" si="24">K48*K55</f>
+        <v>4085.5893750000009</v>
       </c>
       <c r="L49" s="2">
         <f>K49*0.57</f>
-        <v>2347.9137899999996</v>
+        <v>2328.7859437500001</v>
       </c>
       <c r="M49" s="2">
-        <f t="shared" ref="M49:M52" si="22">K49-L49</f>
-        <v>1771.2332100000003</v>
+        <f t="shared" ref="M49:M52" si="25">K49-L49</f>
+        <v>1756.8034312500008</v>
       </c>
       <c r="N49" s="2">
-        <f t="shared" ref="N49:N51" si="23">N48*$N$54</f>
-        <v>1729.5535039999997</v>
+        <f t="shared" ref="N49:N51" si="26">N48*$N$54</f>
+        <v>1722.1065653749997</v>
       </c>
       <c r="O49" s="2">
-        <f t="shared" ref="O49:O52" si="24">N49*0.92</f>
-        <v>1591.1892236799999</v>
+        <f t="shared" ref="O49:O52" si="27">N49*0.92</f>
+        <v>1584.3380401449999</v>
       </c>
       <c r="P49" s="2">
-        <f t="shared" ref="P49:P52" si="25">N49-O49</f>
-        <v>138.36428031999981</v>
+        <f t="shared" ref="P49:P52" si="28">N49-O49</f>
+        <v>137.7685252299998</v>
       </c>
       <c r="R49" s="5"/>
     </row>
@@ -7074,57 +7752,60 @@
         <v>2028</v>
       </c>
       <c r="B50" s="2">
-        <f t="shared" si="18"/>
-        <v>772.40126955999995</v>
+        <f t="shared" si="21"/>
+        <v>829.66149639062405</v>
       </c>
       <c r="C50" s="2">
         <f>B50*0.57</f>
-        <v>440.26872364919996</v>
+        <v>472.9070529426557</v>
       </c>
       <c r="D50" s="2">
+        <f t="shared" si="22"/>
+        <v>356.75444344796836</v>
+      </c>
+      <c r="E50" s="2">
+        <f t="shared" si="23"/>
+        <v>316.09051632672515</v>
+      </c>
+      <c r="F50" s="2">
+        <f t="shared" si="18"/>
+        <v>249.53324132283728</v>
+      </c>
+      <c r="G50" s="2">
         <f t="shared" si="19"/>
-        <v>332.13254591079999</v>
-      </c>
-      <c r="E50" s="2">
+        <v>21.698542723725041</v>
+      </c>
+      <c r="H50" s="2">
         <f t="shared" si="20"/>
-        <v>304.09168301056042</v>
-      </c>
-      <c r="F50" s="2">
-        <f t="shared" si="16"/>
-        <v>254.59027578879977</v>
-      </c>
-      <c r="G50" s="2">
-        <f t="shared" si="17"/>
-        <v>22.138284851200069</v>
-      </c>
-      <c r="H50" s="2"/>
+        <v>70.833333333333258</v>
+      </c>
       <c r="I50" s="4"/>
       <c r="J50">
         <v>2028</v>
       </c>
       <c r="K50" s="2">
-        <f t="shared" si="21"/>
-        <v>4901.7849299999998</v>
+        <f t="shared" si="24"/>
+        <v>4841.423409375001</v>
       </c>
       <c r="L50" s="2">
         <f>K50*0.57</f>
-        <v>2794.0174100999998</v>
+        <v>2759.6113433437504</v>
       </c>
       <c r="M50" s="2">
-        <f t="shared" si="22"/>
-        <v>2107.7675199</v>
+        <f t="shared" si="25"/>
+        <v>2081.8120660312507</v>
       </c>
       <c r="N50" s="2">
-        <f t="shared" si="23"/>
-        <v>2006.2820646399996</v>
+        <f t="shared" si="26"/>
+        <v>1993.338349421562</v>
       </c>
       <c r="O50" s="2">
-        <f t="shared" si="24"/>
-        <v>1845.7794994687997</v>
+        <f t="shared" si="27"/>
+        <v>1833.8712814678372</v>
       </c>
       <c r="P50" s="2">
-        <f t="shared" si="25"/>
-        <v>160.50256517119988</v>
+        <f t="shared" si="28"/>
+        <v>159.46706795372484</v>
       </c>
       <c r="R50" s="5"/>
     </row>
@@ -7133,57 +7814,60 @@
         <v>2029</v>
       </c>
       <c r="B51" s="2">
-        <f t="shared" si="18"/>
-        <v>843.64752607999992</v>
+        <f>($B$52-$B$47)/5+B50</f>
+        <v>919.99449518749873</v>
       </c>
       <c r="C51" s="2">
         <f>B51*0.57</f>
-        <v>480.87908986559989</v>
+        <v>524.39686225687421</v>
       </c>
       <c r="D51" s="2">
+        <f t="shared" si="22"/>
+        <v>395.59763293062451</v>
+      </c>
+      <c r="E51" s="2">
+        <f t="shared" si="23"/>
+        <v>369.90068843563353</v>
+      </c>
+      <c r="F51" s="2">
+        <f t="shared" si="18"/>
+        <v>288.8347268311843</v>
+      </c>
+      <c r="G51" s="2">
         <f t="shared" si="19"/>
-        <v>362.76843621440003</v>
-      </c>
-      <c r="E51" s="2">
+        <v>25.116063202711757</v>
+      </c>
+      <c r="H51" s="2">
         <f t="shared" si="20"/>
-        <v>353.90224401408057</v>
-      </c>
-      <c r="F51" s="2">
-        <f t="shared" si="16"/>
-        <v>295.32471991500779</v>
-      </c>
-      <c r="G51" s="2">
-        <f t="shared" si="17"/>
-        <v>25.680410427391962</v>
-      </c>
-      <c r="H51" s="2"/>
+        <v>70.833333333333258</v>
+      </c>
       <c r="I51" s="4"/>
       <c r="J51">
         <v>2029</v>
       </c>
       <c r="K51" s="2">
         <f>K50*K57</f>
-        <v>5784.1062173999999</v>
+        <v>5688.6725060156268</v>
       </c>
       <c r="L51" s="2">
         <f>K51*0.57</f>
-        <v>3296.9405439179995</v>
+        <v>3242.543328428907</v>
       </c>
       <c r="M51" s="2">
-        <f t="shared" si="22"/>
-        <v>2487.1656734820003</v>
+        <f t="shared" si="25"/>
+        <v>2446.1291775867198</v>
       </c>
       <c r="N51" s="2">
-        <f t="shared" si="23"/>
-        <v>2327.2871949823993</v>
+        <f t="shared" si="26"/>
+        <v>2307.2891394554581</v>
       </c>
       <c r="O51" s="2">
-        <f t="shared" si="24"/>
-        <v>2141.1042193838075</v>
+        <f t="shared" si="27"/>
+        <v>2122.7060082990215</v>
       </c>
       <c r="P51" s="2">
-        <f t="shared" si="25"/>
-        <v>186.18297559859184</v>
+        <f t="shared" si="28"/>
+        <v>184.58313115643659</v>
       </c>
       <c r="R51" s="5"/>
     </row>
@@ -7193,29 +7877,32 @@
       </c>
       <c r="B52" s="2">
         <f>K52-K51</f>
-        <v>914.89378260000012</v>
+        <v>1010.3274939843732</v>
       </c>
       <c r="C52" s="2">
-        <f t="shared" ref="C48:C52" si="26">L52-L51</f>
-        <v>521.48945608200029</v>
+        <f t="shared" ref="C52" si="29">L52-L51</f>
+        <v>575.88667157109285</v>
       </c>
       <c r="D52" s="2">
-        <f t="shared" ref="D48:D52" si="27">M52-M51</f>
-        <v>393.40432651799983</v>
+        <f t="shared" ref="D52" si="30">M52-M51</f>
+        <v>434.44082241328033</v>
       </c>
       <c r="E52" s="2">
-        <f t="shared" ref="E48:E52" si="28">N52-N51</f>
-        <v>403.71280501760066</v>
+        <f t="shared" ref="E52" si="31">N52-N51</f>
+        <v>423.7108605445419</v>
       </c>
       <c r="F52" s="2">
-        <f t="shared" si="16"/>
-        <v>371.41578061619248</v>
+        <f t="shared" si="18"/>
+        <v>389.81399170097848</v>
       </c>
       <c r="G52" s="2">
-        <f t="shared" si="17"/>
-        <v>32.29702440140818</v>
-      </c>
-      <c r="H52" s="2"/>
+        <f t="shared" si="19"/>
+        <v>33.896868843563425</v>
+      </c>
+      <c r="H52" s="2">
+        <f>R27-R26</f>
+        <v>70.833333333333712</v>
+      </c>
       <c r="I52" s="4"/>
       <c r="J52">
         <v>2030</v>
@@ -7229,43 +7916,51 @@
         <v>3818.43</v>
       </c>
       <c r="M52" s="2">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>2880.57</v>
       </c>
       <c r="N52" s="2">
         <v>2731</v>
       </c>
       <c r="O52" s="2">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>2512.52</v>
       </c>
       <c r="P52" s="2">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>218.48000000000002</v>
       </c>
       <c r="R52" s="5"/>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B54" s="2">
+        <f>SUM(B48:B52)</f>
+        <v>4148.3074819531193</v>
+      </c>
+      <c r="E54" s="2">
+        <f>SUM(E48:E52)</f>
+        <v>1580.4525816336259</v>
+      </c>
       <c r="K54">
-        <v>1.23</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="N54">
-        <v>1.1599999999999999</v>
+        <v>1.1575</v>
       </c>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K55">
-        <v>1.22</v>
+        <v>1.2150000000000001</v>
       </c>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K56">
-        <v>1.19</v>
+        <v>1.1850000000000001</v>
       </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K57">
-        <v>1.18</v>
+        <v>1.175</v>
       </c>
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.25">
@@ -7368,7 +8063,7 @@
         <v>17.416499999999999</v>
       </c>
       <c r="E63" s="2">
-        <f t="shared" ref="E63:E76" si="29">SUM(F63:G63)</f>
+        <f t="shared" ref="E63:E76" si="32">SUM(F63:G63)</f>
         <v>39.11</v>
       </c>
       <c r="F63" s="2">
@@ -7392,7 +8087,7 @@
         <v>44.157499999999999</v>
       </c>
       <c r="N63" s="2">
-        <f t="shared" ref="N63:N77" si="30">SUM(O63:P63)</f>
+        <f t="shared" ref="N63:N77" si="33">SUM(O63:P63)</f>
         <v>220.36</v>
       </c>
       <c r="O63" s="2">
@@ -7416,7 +8111,7 @@
         <v>16.286000000000001</v>
       </c>
       <c r="E64" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>46.919999999999995</v>
       </c>
       <c r="F64" s="2">
@@ -7440,7 +8135,7 @@
         <v>60.4435</v>
       </c>
       <c r="N64" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>267.28000000000003</v>
       </c>
       <c r="O64" s="2">
@@ -7464,7 +8159,7 @@
         <v>13.064499999999899</v>
       </c>
       <c r="E65" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>32.92</v>
       </c>
       <c r="F65" s="2">
@@ -7488,7 +8183,7 @@
         <v>73.507999999999996</v>
       </c>
       <c r="N65" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>300.19</v>
       </c>
       <c r="O65" s="2">
@@ -7512,7 +8207,7 @@
         <v>14.433</v>
       </c>
       <c r="E66" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>49.6</v>
       </c>
       <c r="F66" s="2">
@@ -7536,7 +8231,7 @@
         <v>87.940999999999903</v>
       </c>
       <c r="N66" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>349.8</v>
       </c>
       <c r="O66" s="2">
@@ -7560,7 +8255,7 @@
         <v>16.090499999999999</v>
       </c>
       <c r="E67" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>65.59</v>
       </c>
       <c r="F67" s="2">
@@ -7584,7 +8279,7 @@
         <v>104.03149999999999</v>
       </c>
       <c r="N67" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>415.39</v>
       </c>
       <c r="O67" s="2">
@@ -7608,7 +8303,7 @@
         <v>17.7395</v>
       </c>
       <c r="E68" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>52.14</v>
       </c>
       <c r="F68" s="2">
@@ -7632,7 +8327,7 @@
         <v>121.77099999999901</v>
       </c>
       <c r="N68" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>467.53</v>
       </c>
       <c r="O68" s="2">
@@ -7656,7 +8351,7 @@
         <v>32.954500000000003</v>
       </c>
       <c r="E69" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>47.63</v>
       </c>
       <c r="F69" s="2">
@@ -7680,7 +8375,7 @@
         <v>154.73399999999901</v>
       </c>
       <c r="N69" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>515.16</v>
       </c>
       <c r="O69" s="2">
@@ -7704,7 +8399,7 @@
         <v>37.7484999999999</v>
       </c>
       <c r="E70" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>49.66</v>
       </c>
       <c r="F70" s="2">
@@ -7728,7 +8423,7 @@
         <v>192.47399999999999</v>
       </c>
       <c r="N70" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>564.82000000000005</v>
       </c>
       <c r="O70" s="2">
@@ -7752,7 +8447,7 @@
         <v>39.626999999999903</v>
       </c>
       <c r="E71" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>59.03</v>
       </c>
       <c r="F71" s="2">
@@ -7776,7 +8471,7 @@
         <v>232.101</v>
       </c>
       <c r="N71" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>623.85</v>
       </c>
       <c r="O71" s="2">
@@ -7800,7 +8495,7 @@
         <v>55.887499999999903</v>
       </c>
       <c r="E72" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>108.19</v>
       </c>
       <c r="F72" s="2">
@@ -7824,7 +8519,7 @@
         <v>287.99700000000001</v>
       </c>
       <c r="N72" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>732.04</v>
       </c>
       <c r="O72" s="2">
@@ -7848,7 +8543,7 @@
         <v>65.331000000000003</v>
       </c>
       <c r="E73" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>92.81</v>
       </c>
       <c r="F73" s="2">
@@ -7872,7 +8567,7 @@
         <v>353.32799999999997</v>
       </c>
       <c r="N73" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>824.86</v>
       </c>
       <c r="O73" s="2">
@@ -7896,7 +8591,7 @@
         <v>96.959499999999906</v>
       </c>
       <c r="E74" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>76.14</v>
       </c>
       <c r="F74" s="2">
@@ -7920,7 +8615,7 @@
         <v>450.287499999999</v>
       </c>
       <c r="N74" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>900.99</v>
       </c>
       <c r="O74" s="2">
@@ -7944,7 +8639,7 @@
         <v>159.56199999999899</v>
       </c>
       <c r="E75" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>114.57</v>
       </c>
       <c r="F75" s="2">
@@ -7968,7 +8663,7 @@
         <v>609.84100000000001</v>
       </c>
       <c r="N75" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>1015.5699999999999</v>
       </c>
       <c r="O75" s="2">
@@ -7992,7 +8687,7 @@
         <v>181.3475</v>
       </c>
       <c r="E76" s="2">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>115.1</v>
       </c>
       <c r="F76" s="2">
@@ -8016,7 +8711,7 @@
         <v>791.18849999999998</v>
       </c>
       <c r="N76" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>1130.67</v>
       </c>
       <c r="O76" s="2">
@@ -8064,7 +8759,7 @@
         <v>1044.1400000000001</v>
       </c>
       <c r="N77" s="2">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>1285.3399999999999</v>
       </c>
       <c r="O77" s="2">
@@ -8120,15 +8815,15 @@
         <v>1308.3788625000002</v>
       </c>
       <c r="N78" s="2">
-        <f>N77+E78</f>
+        <f t="shared" ref="N78:P82" si="34">N77+E78</f>
         <v>1472.4785999999999</v>
       </c>
       <c r="O78" s="2">
-        <f>O77+F78</f>
+        <f t="shared" si="34"/>
         <v>1358.427512</v>
       </c>
       <c r="P78" s="2">
-        <f>P77+G78</f>
+        <f t="shared" si="34"/>
         <v>114.05108799999998</v>
       </c>
     </row>
@@ -8137,27 +8832,27 @@
         <v>2027</v>
       </c>
       <c r="B79" s="2">
-        <f t="shared" ref="B79:B82" si="31">B78*$B$84</f>
+        <f t="shared" ref="B79:B82" si="35">B78*$B$84</f>
         <v>675.98162500000012</v>
       </c>
       <c r="C79" s="2">
-        <f t="shared" ref="C79:C82" si="32">B79*0.57</f>
+        <f t="shared" ref="C79:C82" si="36">B79*0.57</f>
         <v>385.30952625000003</v>
       </c>
       <c r="D79" s="2">
-        <f t="shared" ref="D79:D82" si="33">B79-C79</f>
+        <f t="shared" ref="D79:D82" si="37">B79-C79</f>
         <v>290.67209875000009</v>
       </c>
       <c r="E79" s="2">
-        <f t="shared" ref="E79:E82" si="34">E78*$E$84</f>
+        <f t="shared" ref="E79:E82" si="38">E78*$E$84</f>
         <v>226.43770599999999</v>
       </c>
       <c r="F79" s="2">
-        <f t="shared" ref="F79:F82" si="35">E79*0.92</f>
+        <f t="shared" ref="F79:F82" si="39">E79*0.92</f>
         <v>208.32268952000001</v>
       </c>
       <c r="G79" s="2">
-        <f t="shared" ref="G79:G82" si="36">E79-F79</f>
+        <f t="shared" ref="G79:G82" si="40">E79-F79</f>
         <v>18.11501647999998</v>
       </c>
       <c r="H79" s="2"/>
@@ -8166,27 +8861,27 @@
         <v>2027</v>
       </c>
       <c r="K79" s="2">
-        <f t="shared" ref="K79" si="37">K78+B79</f>
+        <f t="shared" ref="K79" si="41">K78+B79</f>
         <v>3685.6403749999999</v>
       </c>
       <c r="L79" s="2">
-        <f t="shared" ref="L79:L82" si="38">L78+C79</f>
+        <f t="shared" ref="L79:L82" si="42">L78+C79</f>
         <v>2086.5894137499999</v>
       </c>
       <c r="M79" s="2">
-        <f t="shared" ref="M79:M82" si="39">K79-L79</f>
+        <f t="shared" ref="M79:M82" si="43">K79-L79</f>
         <v>1599.05096125</v>
       </c>
       <c r="N79" s="2">
-        <f>N78+E79</f>
+        <f t="shared" si="34"/>
         <v>1698.9163059999998</v>
       </c>
       <c r="O79" s="2">
-        <f>O78+F79</f>
+        <f t="shared" si="34"/>
         <v>1566.75020152</v>
       </c>
       <c r="P79" s="2">
-        <f>P78+G79</f>
+        <f t="shared" si="34"/>
         <v>132.16610447999994</v>
       </c>
     </row>
@@ -8195,27 +8890,27 @@
         <v>2028</v>
       </c>
       <c r="B80" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="35"/>
         <v>743.57978750000018</v>
       </c>
       <c r="C80" s="2">
-        <f t="shared" si="32"/>
+        <f t="shared" si="36"/>
         <v>423.84047887500009</v>
       </c>
       <c r="D80" s="2">
-        <f t="shared" si="33"/>
+        <f t="shared" si="37"/>
         <v>319.73930862500009</v>
       </c>
       <c r="E80" s="2">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>273.98962425999997</v>
       </c>
       <c r="F80" s="2">
-        <f t="shared" si="35"/>
+        <f t="shared" si="39"/>
         <v>252.0704543192</v>
       </c>
       <c r="G80" s="2">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>21.919169940799975</v>
       </c>
       <c r="H80" s="2"/>
@@ -8228,23 +8923,23 @@
         <v>4429.2201624999998</v>
       </c>
       <c r="L80" s="2">
-        <f t="shared" si="38"/>
+        <f t="shared" si="42"/>
         <v>2510.4298926249999</v>
       </c>
       <c r="M80" s="2">
-        <f t="shared" si="39"/>
+        <f t="shared" si="43"/>
         <v>1918.7902698749999</v>
       </c>
       <c r="N80" s="2">
-        <f>N79+E80</f>
+        <f t="shared" si="34"/>
         <v>1972.9059302599999</v>
       </c>
       <c r="O80" s="2">
-        <f>O79+F80</f>
+        <f t="shared" si="34"/>
         <v>1818.8206558392001</v>
       </c>
       <c r="P80" s="2">
-        <f>P79+G80</f>
+        <f t="shared" si="34"/>
         <v>154.08527442079992</v>
       </c>
     </row>
@@ -8253,27 +8948,27 @@
         <v>2029</v>
       </c>
       <c r="B81" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="35"/>
         <v>817.93776625000021</v>
       </c>
       <c r="C81" s="2">
-        <f t="shared" si="32"/>
+        <f t="shared" si="36"/>
         <v>466.22452676250009</v>
       </c>
       <c r="D81" s="2">
-        <f t="shared" si="33"/>
+        <f t="shared" si="37"/>
         <v>351.71323948750012</v>
       </c>
       <c r="E81" s="2">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>331.52744535459993</v>
       </c>
       <c r="F81" s="2">
-        <f t="shared" si="35"/>
+        <f t="shared" si="39"/>
         <v>305.00524972623197</v>
       </c>
       <c r="G81" s="2">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>26.522195628367967</v>
       </c>
       <c r="H81" s="2"/>
@@ -8286,23 +8981,23 @@
         <v>5247.1579287499999</v>
       </c>
       <c r="L81" s="2">
-        <f t="shared" si="38"/>
+        <f t="shared" si="42"/>
         <v>2976.6544193874997</v>
       </c>
       <c r="M81" s="2">
-        <f t="shared" si="39"/>
+        <f t="shared" si="43"/>
         <v>2270.5035093625002</v>
       </c>
       <c r="N81" s="2">
-        <f>N80+E81</f>
+        <f t="shared" si="34"/>
         <v>2304.4333756145998</v>
       </c>
       <c r="O81" s="2">
-        <f>O80+F81</f>
+        <f t="shared" si="34"/>
         <v>2123.8259055654321</v>
       </c>
       <c r="P81" s="2">
-        <f>P80+G81</f>
+        <f t="shared" si="34"/>
         <v>180.60747004916789</v>
       </c>
     </row>
@@ -8311,27 +9006,27 @@
         <v>2030</v>
       </c>
       <c r="B82" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="35"/>
         <v>899.73154287500029</v>
       </c>
       <c r="C82" s="2">
-        <f t="shared" si="32"/>
+        <f t="shared" si="36"/>
         <v>512.84697943875017</v>
       </c>
       <c r="D82" s="2">
-        <f t="shared" si="33"/>
+        <f t="shared" si="37"/>
         <v>386.88456343625012</v>
       </c>
       <c r="E82" s="2">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>401.14820887906592</v>
       </c>
       <c r="F82" s="2">
-        <f t="shared" si="35"/>
+        <f t="shared" si="39"/>
         <v>369.05635216874066</v>
       </c>
       <c r="G82" s="2">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>32.09185671032526</v>
       </c>
       <c r="H82" s="2"/>
@@ -8344,23 +9039,23 @@
         <v>5694.15</v>
       </c>
       <c r="L82" s="2">
-        <f t="shared" si="38"/>
+        <f t="shared" si="42"/>
         <v>3489.5013988262499</v>
       </c>
       <c r="M82" s="2">
-        <f t="shared" si="39"/>
+        <f t="shared" si="43"/>
         <v>2204.6486011737497</v>
       </c>
       <c r="N82" s="2">
-        <f>N81+E82</f>
+        <f t="shared" si="34"/>
         <v>2705.5815844936656</v>
       </c>
       <c r="O82" s="2">
-        <f>O81+F82</f>
+        <f t="shared" si="34"/>
         <v>2492.8822577341725</v>
       </c>
       <c r="P82" s="2">
-        <f>P81+G82</f>
+        <f t="shared" si="34"/>
         <v>212.69932675949315</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Clean tripling workbook artifacts
</commit_message>
<xml_diff>
--- a/tripling_beta/tripling.xlsx
+++ b/tripling_beta/tripling.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Documents\GitHub\GIPT\tripling_beta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD457CC-2C93-4D4E-B43E-71A6A41D2259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{097C5675-4190-4277-9625-F8A06871B357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{64387DDE-4ECD-4D35-9D9B-650204D19CA6}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="30">
   <si>
     <t>Historical annual capacity additions</t>
   </si>
@@ -6836,6 +6836,9 @@
       <c r="G31" t="s">
         <v>6</v>
       </c>
+      <c r="H31" t="s">
+        <v>11</v>
+      </c>
       <c r="K31" t="s">
         <v>2</v>
       </c>

</xml_diff>